<commit_message>
Tentando atualizar a lista
</commit_message>
<xml_diff>
--- a/3D/base_de_dados.xlsx
+++ b/3D/base_de_dados.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PC- lixos\Downloads-24-11-2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9CD3D54-DD64-4421-85D1-09A52FAD685D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDA024D2-6AB5-4573-839F-6CE930EEB797}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1464" yWindow="1464" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{F08DF800-D7FB-4182-BEE8-B029C50FA673}"/>
+    <workbookView xWindow="5856" yWindow="1428" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{F08DF800-D7FB-4182-BEE8-B029C50FA673}"/>
   </bookViews>
   <sheets>
     <sheet name="Associa" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="17">
   <si>
     <t>CÓDIGO</t>
   </si>
@@ -78,13 +78,16 @@
     <t>Descrição</t>
   </si>
   <si>
-    <t>Aterramento - Haste de aterramento - cobreada - 5/8\" x 2,40m</t>
-  </si>
-  <si>
-    <t>Aterramento - Conector tipo \"U\" - 5/8\"</t>
-  </si>
-  <si>
     <t>Aterramento - Caixa de inspeção - Polipropileno - Ø300x400mm</t>
+  </si>
+  <si>
+    <t>Aterramento - Haste de aterramento - cobreada - 5/8" x 2,40m</t>
+  </si>
+  <si>
+    <t>Aterramento - Conector tipo "U" - 5/8"</t>
+  </si>
+  <si>
+    <t>Aterramento - Caixa de inspeção - Polipropileno - Ø300x300mm</t>
   </si>
 </sst>
 </file>
@@ -469,22 +472,22 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizando a base de dados
</commit_message>
<xml_diff>
--- a/3D/base_de_dados.xlsx
+++ b/3D/base_de_dados.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PC- lixos\Downloads-24-11-2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AED07F2D-F782-4E20-B30E-56B31EA4F3A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E47302E3-DAAE-4318-BE66-E6023BFA26F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" xr2:uid="{F08DF800-D7FB-4182-BEE8-B029C50FA673}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{F08DF800-D7FB-4182-BEE8-B029C50FA673}"/>
   </bookViews>
   <sheets>
     <sheet name="Associa" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="195">
   <si>
     <t>CÓDIGO</t>
   </si>
@@ -463,6 +463,165 @@
   </si>
   <si>
     <t>INTERRUPTOR SIMPLES (1 MÓDULO), 10A/250V, INCLUINDO SUPORTE E PLACA - FORNECIMENTO E INSTALAÇÃO. AF_03/2023</t>
+  </si>
+  <si>
+    <t>Eletrocalha furada tipo U pré-galv. quen - Suporte vertical - 70x81mm</t>
+  </si>
+  <si>
+    <t>Comp 742</t>
+  </si>
+  <si>
+    <t>SUPORTE VERTICAL - 70X81MM (COMPOSIÇÃO DE REFERÊNCIA: SINAPI 97274 - 09/2022)</t>
+  </si>
+  <si>
+    <t>Eletrocalha furada tipo U pré-galv. quen - Suporte vertical - 120x175mm</t>
+  </si>
+  <si>
+    <t>Comp 822</t>
+  </si>
+  <si>
+    <t>SUPORTE VERTICAL 120X175MM - (COMPOSIÇÃO DE REFERÊNCIA: SINAPI 97274 - 09/2022)</t>
+  </si>
+  <si>
+    <t>Eletrocalha furada tipo U pré-galv. quen - Suporte vertical - 120x204mm</t>
+  </si>
+  <si>
+    <t>Comp 797</t>
+  </si>
+  <si>
+    <t>SUPORTE VERTICAL 120X204MM - (COMPOSIÇÃO DE REFERÊNCIA: SINAPI 97274 - 09/2022)</t>
+  </si>
+  <si>
+    <t>Eletrocalha furada tipo U pré-galv. quen - Suporte vertical - 120x146mm</t>
+  </si>
+  <si>
+    <t>Comp 1397</t>
+  </si>
+  <si>
+    <t>SUPORTE VERTICAL 120X146MM - (COMPOSIÇÃO DE REFERÊNCIA: SINAPI 97274 - 09/2022)</t>
+  </si>
+  <si>
+    <t>Acessórios Perfilados perfurados - Curva horizontal 90° - 38x38mm</t>
+  </si>
+  <si>
+    <t>Comp 330</t>
+  </si>
+  <si>
+    <t>CURVA HORIZONTAL 90° PARA PERFILADOS PERFURADOS 38x38mm (COMPOSIÇÃO DE REFERÊNCIA: SINAPI 97274 - 09/2022)</t>
+  </si>
+  <si>
+    <t>Dispositivo de Proteção - Dispositivo de proteção contra surto - 175 V - 25 KA</t>
+  </si>
+  <si>
+    <t>DISPOSITIVO DE PROTEÇÃO CONTRA SURTO DPS 25KA - 175V (COMPOSIÇÃO DE REFERÊNCIA: ORSE 13150 - 05/2023)</t>
+  </si>
+  <si>
+    <t>Comp 785</t>
+  </si>
+  <si>
+    <t>Dispositivo de Proteção - Dispositivo de proteção contra surto - 175 V - 80 KA</t>
+  </si>
+  <si>
+    <t>DISPOSITIVO DE PROTEÇÃO CONTRA SURTO DPS 80KA - 175V (COMPOSIÇÃO DE REFERÊNCIA: ORSE 9041 - 05/2023)</t>
+  </si>
+  <si>
+    <t>Comp 1536</t>
+  </si>
+  <si>
+    <t>Dispositivo de Proteção - Dispositivo de proteção contra surto - 175 V - 8 KA</t>
+  </si>
+  <si>
+    <t>DISPOSITIVO DE PROTEÇÃO CONTRA SURTO DPS 8KA - 175V (COMPOSIÇÃO DE REFERÊNCIA: ORSE 13150 - 05/2023)</t>
+  </si>
+  <si>
+    <t>Comp 1629</t>
+  </si>
+  <si>
+    <t>Dispositivo de Proteção - Disjuntor unipolar termomagnético - 220 V/127 V - DIN - Curva B - 20 A - 5 kA</t>
+  </si>
+  <si>
+    <t>Dispositivo Elétrico - embutido - Placa 2x4" - Interruptor simples &amp; paralelo - 2 teclas</t>
+  </si>
+  <si>
+    <t>INTERRUPTOR SIMPLES (1 MÓDULO) COM INTERRUPTOR PARALELO (1 MÓDULO), 10A/250V, INCLUINDO SUPORTE E PLACA - FORNECIMENTO E INSTALAÇÃO. AF_03/2023</t>
+  </si>
+  <si>
+    <t>Dispositivo Elétrico - embutido - S/ placa - Tomada hexagonal - NBR 14136 - 2 - 2P+T 10A - Média</t>
+  </si>
+  <si>
+    <t>TOMADA MÉDIA DE EMBUTIR (2 MÓDULOS), 2P+T 10 A, INCLUINDO SUPORTE E PLACA - FORNECIMENTO E INSTALAÇÃO. AF_03/2023</t>
+  </si>
+  <si>
+    <t>Dispositivo Elétrico - embutido - S/ placa - Tomada hexagonal - NBR 14136 - 2P+T 10A - Média</t>
+  </si>
+  <si>
+    <t>TOMADA MÉDIA DE EMBUTIR (1 MÓDULO), 2P+T 10 A, INCLUINDO SUPORTE E PLACA - FORNECIMENTO E INSTALAÇÃO. AF_03/2023</t>
+  </si>
+  <si>
+    <t>Eletrocalha furada tipo U pré-galv. quen - Curva horizontal 90° - 300x100mm chapa 18</t>
+  </si>
+  <si>
+    <t>Comp 453</t>
+  </si>
+  <si>
+    <t>CURVA HORIZONTAL 90º PARA ELETROCALHA, LISA OU PERFURADA EM AÇO GALVANIZADO, LARGURA DE 300MM E ALTURA DE 100MM - FORNECIMENTO E INSTALAÇÃO (COMPOSIÇÃO DE REFERÊNCIA: SINAPI 97278 - 02/2023)</t>
+  </si>
+  <si>
+    <t>Eletrocalha furada tipo U pré-galv. quen - T horizontal 90° - 300x100mm chapa 18</t>
+  </si>
+  <si>
+    <t>TE HORIZONTAL PARA ELETROCALHA 300X100MM (COMPOSIÇÃO DE REFERÊNCIA: SINAPI 97315 - 02/2023)</t>
+  </si>
+  <si>
+    <t>Comp 463</t>
+  </si>
+  <si>
+    <t>Comp 461</t>
+  </si>
+  <si>
+    <t>TERMINAL 300 X 100 PARA ELETROCALHA (COMPOSIÇÃO REFERÊNCIA: 12611 ORSE 05/23)</t>
+  </si>
+  <si>
+    <t>Eletrocalha furada tipo U pré-galv. quen - Terminal - 300x100mm chapa 18</t>
+  </si>
+  <si>
+    <t>Eletrocalha furada tipo U pré-galv. quen - Terminal - 200x100mm chapa 18</t>
+  </si>
+  <si>
+    <t>Comp 460</t>
+  </si>
+  <si>
+    <t>TERMINAL 200 X 100 PARA ELETROCALHA (COMPOSIÇÃO REFERÊNCIA: 12611 ORSE 05/23)</t>
+  </si>
+  <si>
+    <t>Eletrocalha furada tipo U pré-galv. quen - Terminal - 100x100mm chapa 18</t>
+  </si>
+  <si>
+    <t>Comp 458</t>
+  </si>
+  <si>
+    <t>TERMINAL 100 X 100 PARA ELETROCALHA (COMPOSIÇÃO REFERÊNCIA: 12611 ORSE 05/23)</t>
+  </si>
+  <si>
+    <t>.S.O.S CAIXAS - 80x80 - piso - CAIXA DE PASSAGEM EM ALVENARIA, DIM.: 80x80cm, COM TAMPA DE FERRO FUNDIDO T-33. FORNECIMENTO E INSTALAÇÃO.</t>
+  </si>
+  <si>
+    <t>CAIXA ENTERRADA ELÉTRICA RETANGULAR, EM ALVENARIA COM TIJOLOS CERÂMICOS MACIÇOS, FUNDO COM BRITA, DIMENSÕES INTERNAS: 0,8X0,8X0,6 M. AF_12/2020</t>
+  </si>
+  <si>
+    <t>.S.O.S CAIXA DE PASSAGEM - EMBUTIR NO PISO - Alvenaria - 60x60x60 cm</t>
+  </si>
+  <si>
+    <t>CAIXA ENTERRADA ELÉTRICA RETANGULAR, EM ALVENARIA COM TIJOLOS CERÂMICOS MACIÇOS, FUNDO COM BRITA, DIMENSÕES INTERNAS: 0,6X0,6X0,6 M. AF_12/2020</t>
+  </si>
+  <si>
+    <t>Intelbras - Equipamentos de Rede e Rack - Rack de Piso - 16U unc 19” x 570mm RPD 1657</t>
+  </si>
+  <si>
+    <t>Comp 226</t>
+  </si>
+  <si>
+    <t>RACK ABERTO PADRÃO 19" 16U  (COMPOSIÇÃO DE REFERÊNCIA: SBC 059085 - 06/2022)</t>
   </si>
 </sst>
 </file>
@@ -849,7 +1008,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A62C0A3C-3A73-4C24-9726-9CC231B21D7A}">
-  <dimension ref="A1:B74"/>
+  <dimension ref="A1:B94"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="96.77734375" style="3" bestFit="1" customWidth="1"/>
@@ -1354,7 +1513,7 @@
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A63" s="3" t="s">
-        <v>114</v>
+        <v>166</v>
       </c>
       <c r="B63" s="1" t="s">
         <v>7</v>
@@ -1362,7 +1521,7 @@
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A64" s="3" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B64" s="1" t="s">
         <v>7</v>
@@ -1370,7 +1529,7 @@
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A65" s="3" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B65" s="1" t="s">
         <v>7</v>
@@ -1378,7 +1537,7 @@
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A66" s="3" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B66" s="1" t="s">
         <v>7</v>
@@ -1386,7 +1545,7 @@
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A67" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B67" s="1" t="s">
         <v>7</v>
@@ -1394,7 +1553,7 @@
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A68" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B68" s="1" t="s">
         <v>7</v>
@@ -1402,7 +1561,7 @@
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A69" s="3" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B69" s="1" t="s">
         <v>7</v>
@@ -1410,7 +1569,7 @@
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A70" s="3" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B70" s="1" t="s">
         <v>7</v>
@@ -1418,7 +1577,7 @@
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A71" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B71" s="1" t="s">
         <v>7</v>
@@ -1426,7 +1585,7 @@
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A72" s="3" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B72" s="1" t="s">
         <v>7</v>
@@ -1434,7 +1593,7 @@
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A73" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B73" s="1" t="s">
         <v>7</v>
@@ -1442,9 +1601,169 @@
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A74" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A75" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="B74" s="1" t="s">
+      <c r="B75" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A76" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A77" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A78" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A79" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A80" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A81" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A82" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A83" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A84" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A85" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A86" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A87" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A88" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A89" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A90" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A91" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A92" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A93" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A94" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="B94" s="1" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1455,7 +1774,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DACEE6F-7DD5-4F5D-8CC1-2F57EE446892}">
-  <dimension ref="A1:D74"/>
+  <dimension ref="A1:D94"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.109375" style="2" bestFit="1" customWidth="1"/>
@@ -2334,13 +2653,13 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63" s="2">
-        <v>93654</v>
+        <v>93655</v>
       </c>
       <c r="B63" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>7</v>
@@ -2348,13 +2667,13 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64" s="2">
-        <v>93663</v>
+        <v>93654</v>
       </c>
       <c r="B64" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>7</v>
@@ -2362,13 +2681,13 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65" s="2">
-        <v>93661</v>
+        <v>93663</v>
       </c>
       <c r="B65" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>7</v>
@@ -2376,13 +2695,13 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66" s="2">
-        <v>93654</v>
+        <v>93661</v>
       </c>
       <c r="B66" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>7</v>
@@ -2390,27 +2709,27 @@
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67" s="2">
+        <v>93654</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A68" s="2">
         <v>93671</v>
       </c>
-      <c r="B67" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C67" s="3" t="s">
+      <c r="B68" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C68" s="3" t="s">
         <v>122</v>
-      </c>
-      <c r="D67" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A68" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="B68" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C68" s="3" t="s">
-        <v>125</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>7</v>
@@ -2418,13 +2737,13 @@
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B69" s="3" t="s">
         <v>69</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>7</v>
@@ -2432,13 +2751,13 @@
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B70" s="3" t="s">
         <v>69</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D70" s="2" t="s">
         <v>7</v>
@@ -2446,57 +2765,337 @@
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B71" s="3" t="s">
         <v>69</v>
       </c>
       <c r="C71" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A72" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C72" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="D71" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A72" s="2">
+      <c r="D72" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A73" s="2">
         <v>91961</v>
       </c>
-      <c r="B72" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C72" s="3" t="s">
+      <c r="B73" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C73" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="D72" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A73" s="2" t="s">
+      <c r="D73" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A74" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B73" s="3" t="s">
+      <c r="B74" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="C73" s="3" t="s">
+      <c r="C74" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="D73" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A74" s="2">
+      <c r="D74" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A75" s="2">
         <v>91953</v>
       </c>
-      <c r="B74" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C74" s="3" t="s">
+      <c r="B75" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C75" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="D74" s="2" t="s">
+      <c r="D75" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A76" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C76" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A77" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B77" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C77" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A78" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A79" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A80" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B80" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C80" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A81" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C81" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A82" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C82" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A83" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="B83" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C83" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A84" s="2">
+        <v>91957</v>
+      </c>
+      <c r="B84" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C84" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A85" s="2">
+        <v>92004</v>
+      </c>
+      <c r="B85" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C85" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A86" s="2">
+        <v>91996</v>
+      </c>
+      <c r="B86" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C86" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A87" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B87" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C87" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A88" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B88" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C88" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A89" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="B89" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C89" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A90" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="B90" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C90" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A91" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="B91" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C91" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A92" s="2">
+        <v>97889</v>
+      </c>
+      <c r="B92" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C92" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A93" s="2">
+        <v>97888</v>
+      </c>
+      <c r="B93" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C93" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="D93" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A94" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B94" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C94" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="D94" s="2" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Tentando melhorar a lista
</commit_message>
<xml_diff>
--- a/3D/base_de_dados.xlsx
+++ b/3D/base_de_dados.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PC- lixos\Downloads-24-11-2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82A97847-D785-4D34-8431-DDE541EF4990}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1A0422F-C701-42A9-B702-CBB8BF6D601E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{F08DF800-D7FB-4182-BEE8-B029C50FA673}"/>
+    <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" xr2:uid="{F08DF800-D7FB-4182-BEE8-B029C50FA673}"/>
   </bookViews>
   <sheets>
     <sheet name="Associa" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="265">
   <si>
     <t>CÓDIGO</t>
   </si>
@@ -697,6 +697,141 @@
   </si>
   <si>
     <t>REPETIDOR DE SINAL (COMPOSIÇÃO DE REFERÊNCIA: CPOS/CDHU: 61.15.140 09/2024)</t>
+  </si>
+  <si>
+    <t>Acessórios Cabeamento - Ótico - Extensão ótica MM - 2 fibras - Conetor ST</t>
+  </si>
+  <si>
+    <t>Comp 1183</t>
+  </si>
+  <si>
+    <t>EXTENSÃO ÓPTICA LC/SC MM 2FO (COMPOSIÇÃO DE REFERÊNCIA: 13596 ORSE 05/2025)</t>
+  </si>
+  <si>
+    <t>Acessórios Cabeamento - Metálico - Switch - 10/100 - BaseTX - 48 portas</t>
+  </si>
+  <si>
+    <t>Comp 1613</t>
+  </si>
+  <si>
+    <t>SWITCH 48 PORTAS (COMPOSIÇÃO DE REFERÊNCIA: SBC 059085 - 06/2022)</t>
+  </si>
+  <si>
+    <t>Comp 371</t>
+  </si>
+  <si>
+    <t>TE HORIZONTAL PARA ELETROCALHA 50X50 (COMPOSIÇÃO DE REFERÊNCIA: SINAPI 97274 - 09/2022)</t>
+  </si>
+  <si>
+    <t>Eletrocalha furada tipo U pré-galv. quen - T horizontal 90° - 50x50mm chapa 18</t>
+  </si>
+  <si>
+    <t>Eletrocalha furada tipo U pré-galv. quen - Terminal - 50x50mm chapa 18</t>
+  </si>
+  <si>
+    <t>Comp 1608</t>
+  </si>
+  <si>
+    <t>TERMINAL 50 X 50 PARA ELETROCALHA (COMPOSIÇÃO REFERÊNCIA: 12611 ORSE 05/23)</t>
+  </si>
+  <si>
+    <t>Eletrocalha furada tipo U pré-galv. quen - Acessórios para eletrocalha - Saída dupla para eletroduto</t>
+  </si>
+  <si>
+    <t>Comp 451</t>
+  </si>
+  <si>
+    <t>SAIDA HORIZONTAL DUPLA PARA ELETRODUTO (COMPOSIÇÃO DE REFERÊNCIA: 063756 SBC 05/2024)</t>
+  </si>
+  <si>
+    <t>Acessórios Cabeamento - Ótico - Conetor - ST</t>
+  </si>
+  <si>
+    <t>Comp 1181</t>
+  </si>
+  <si>
+    <t>CONECTOR ÓPTICO ST (COMPOSIÇÃO DE REFERÊNCIA: 059566 SBC 05/2025)</t>
+  </si>
+  <si>
+    <t>Eletrocalha furada tipo U pré-galv. quen - Curva horizontal 90° - 50x50mm chapa 18</t>
+  </si>
+  <si>
+    <t>Comp 516</t>
+  </si>
+  <si>
+    <t>CURVA HORIZONTAL 90º PARA ELETROCALHA, LISA OU PERFURADA EM AÇO GALVANIZADO, LARGURA DE 50MM E ALTURA DE 50MM - FORNECIMENTO E INSTALAÇÃO (COMPOSIÇÃO DE REFERÊNCIA: SINAPI 97278 - 02/2023)</t>
+  </si>
+  <si>
+    <t>Eletrocalha furada tipo U pré-galv. quen - Curva vertical externa 90° - 50x50mm chapa 18</t>
+  </si>
+  <si>
+    <t>Comp 885</t>
+  </si>
+  <si>
+    <t>CURVA VERTICAL EXTERNA 90º PARA ELETROCALHA PERFURADA OU LISA,50X50MM. (REFERÊNCIA: EMOP 15.018.0630-0)</t>
+  </si>
+  <si>
+    <t>Eletrocalha furada tipo U pré-galv. quen - Curva vertical interna 90° - 50x50mm chapa 18</t>
+  </si>
+  <si>
+    <t>Comp 884</t>
+  </si>
+  <si>
+    <t>CURVA VERTICAL INTERNA 90º PARA ELETROCALHA PERFURADA OU LISA,50X50MM. (REFERÊNCIA: EMOP 15.018.0688-0)</t>
+  </si>
+  <si>
+    <t>Acessórios Cabeamento - Metálico - Patch panel - 48 posições</t>
+  </si>
+  <si>
+    <t>Comp 919</t>
+  </si>
+  <si>
+    <t>PATCH PANEL 48 PORTAS CAT 6 T568 T568a/b FURUKAWA (REFERÊNCIA: SBC 059439 01/2025)</t>
+  </si>
+  <si>
+    <t>Acessórios Cabeamento - Metálico - Patch panel - 24 posições</t>
+  </si>
+  <si>
+    <t>Comp 1990</t>
+  </si>
+  <si>
+    <t>PATCH PANEL 24 PORTAS CAT 6 T568 T568a/b FURUKAWA (REFERÊNCIA: SBC 059439 01/2025)</t>
+  </si>
+  <si>
+    <t>Acessórios Perfilados perfurados - T horizontal 90° - 38x38mm</t>
+  </si>
+  <si>
+    <t>Comp 796</t>
+  </si>
+  <si>
+    <t>TE HORIZONTAL PARA ELETROCALHA 38x38 (COMPOSIÇÃO DE REFERÊNCIA: SINAPI 97274 - 09/2022)</t>
+  </si>
+  <si>
+    <t>Eletrocalha furada tipo U pré-galv. quen - Tala plana perfurada - 50mm</t>
+  </si>
+  <si>
+    <t>Comp 455</t>
+  </si>
+  <si>
+    <t>TALA PLANA PERFURADA PARA ELETROCALHA 50MM METALICA (COMPOSIÇÃO DE REFERÊNCIA: 9524 ORSE 03/2024)</t>
+  </si>
+  <si>
+    <t>.S.O.S CFTV e Segurança - CFTV - IP/POE - Câmera de Segurança tipo Bullet 90° IP66</t>
+  </si>
+  <si>
+    <t>Comp 1159</t>
+  </si>
+  <si>
+    <t>CÂMERA DE MONITORAMENTO COM ATÉ 25 METROS DE ALCANCE TIPO BULLET - FORNECIMENTO E INSTALAÇÃO. AF_09/2024 (BASEADO EM SINAPI 97603 03/2025)</t>
+  </si>
+  <si>
+    <t>Eletrocalha furada tipo U pré-galv. quen - Acessórios para eletrocalha - Saída horizontal para eletroduto</t>
+  </si>
+  <si>
+    <t>CONDULETE DE ALUMÍNIO, TIPO X, PARA ELETRODUTO DE AÇO GALVANIZADO DN 32 MM (1 1/4&amp;#39;&amp;#39;), APARENTE - FORNECIMENTO E INSTALAÇÃO. AF_10/2022</t>
+  </si>
+  <si>
+    <t>.S.O.S CAIXAS - Conduletes - CAIXA DE DERIVAÇÃO EM ALUMÍNIO SILÍCIO INJETADO, CONDULETE DE Ø1". FORNECIMENTO E INSTALAÇÃO.</t>
   </si>
 </sst>
 </file>
@@ -1083,7 +1218,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A62C0A3C-3A73-4C24-9726-9CC231B21D7A}">
-  <dimension ref="A1:B103"/>
+  <dimension ref="A1:B119"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="96.77734375" style="3" bestFit="1" customWidth="1"/>
@@ -1914,6 +2049,134 @@
         <v>7</v>
       </c>
     </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A104" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A105" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A106" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A107" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A108" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A109" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A110" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A111" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A112" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A113" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A114" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A115" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A116" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A117" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A118" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="B118" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A119" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="B119" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
@@ -1921,7 +2184,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DACEE6F-7DD5-4F5D-8CC1-2F57EE446892}">
-  <dimension ref="A1:D103"/>
+  <dimension ref="A1:D119"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.109375" style="2" bestFit="1" customWidth="1"/>
@@ -3372,6 +3635,230 @@
         <v>7</v>
       </c>
     </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A104" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B104" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C104" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A105" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B105" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C105" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="D105" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A106" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B106" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C106" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="D106" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A107" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="B107" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C107" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="D107" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A108" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="B108" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C108" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="D108" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A109" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="B109" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C109" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="D109" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A110" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B110" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C110" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="D110" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A111" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="B111" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C111" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="D111" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A112" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="B112" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C112" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="D112" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A113" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="B113" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C113" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D113" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A114" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="B114" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C114" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="D114" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A115" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="B115" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C115" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="D115" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A116" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B116" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C116" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="D116" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A117" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="B117" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C117" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="D117" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A118" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="B118" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C118" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="D118" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A119" s="2">
+        <v>95803</v>
+      </c>
+      <c r="B119" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C119" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="D119" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
Tentando melhorar a lista de materiais
</commit_message>
<xml_diff>
--- a/3D/base_de_dados.xlsx
+++ b/3D/base_de_dados.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PC- lixos\Downloads-24-11-2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1A0422F-C701-42A9-B702-CBB8BF6D601E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F575C74C-F953-4BAB-8447-A2622DB055FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" xr2:uid="{F08DF800-D7FB-4182-BEE8-B029C50FA673}"/>
+    <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{F08DF800-D7FB-4182-BEE8-B029C50FA673}"/>
   </bookViews>
   <sheets>
     <sheet name="Associa" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="275">
   <si>
     <t>CÓDIGO</t>
   </si>
@@ -832,6 +832,36 @@
   </si>
   <si>
     <t>.S.O.S CAIXAS - Conduletes - CAIXA DE DERIVAÇÃO EM ALUMÍNIO SILÍCIO INJETADO, CONDULETE DE Ø1". FORNECIMENTO E INSTALAÇÃO.</t>
+  </si>
+  <si>
+    <t>Acessórios Cabeamento - Metálico - Conector - RJ45 - CM8v - Cat 6, para Patch Panel - Keystone</t>
+  </si>
+  <si>
+    <t>Comp 349</t>
+  </si>
+  <si>
+    <t>CONECTOR RJ-45 CAT. 6 (COMPOSIÇÃO DE REFERÊNCIA: AGETOP CIVIL 071026 - 04/2022)</t>
+  </si>
+  <si>
+    <t>Acessórios Cabeamento - Metálico - Conector - RJ45 - CM8v</t>
+  </si>
+  <si>
+    <t>Acessórios Cabeamento - Metálico - Conector - RJ45 - Blindado - Cat 6</t>
+  </si>
+  <si>
+    <t>Acessórios Cabeamento - Metálico - Plugue - RJ45 - CM8v - Cat 6</t>
+  </si>
+  <si>
+    <t>Comp 1267</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CONECTOR  MACHO, PARA RJ45  CAT 6 - REF. SBC (061359)</t>
+  </si>
+  <si>
+    <t>Acessórios Cabeamento - Metálico - Conector - 110 IDC - 4 pares</t>
+  </si>
+  <si>
+    <t>Acessórios Cabeamento - Metálico - Plugue - 110 IDC - 4 pares</t>
   </si>
 </sst>
 </file>
@@ -1218,7 +1248,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A62C0A3C-3A73-4C24-9726-9CC231B21D7A}">
-  <dimension ref="A1:B119"/>
+  <dimension ref="A1:B125"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="96.77734375" style="3" bestFit="1" customWidth="1"/>
@@ -2177,6 +2207,54 @@
         <v>7</v>
       </c>
     </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A120" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A121" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="B121" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A122" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A123" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A124" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A125" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="B125" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
@@ -2184,7 +2262,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DACEE6F-7DD5-4F5D-8CC1-2F57EE446892}">
-  <dimension ref="A1:D119"/>
+  <dimension ref="A1:D125"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.109375" style="2" bestFit="1" customWidth="1"/>
@@ -3859,6 +3937,90 @@
         <v>7</v>
       </c>
     </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A120" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="B120" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C120" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="D120" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A121" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="B121" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C121" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="D121" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A122" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="B122" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C122" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="D122" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A123" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="B123" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C123" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="D123" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A124" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="B124" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C124" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="D124" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A125" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="B125" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C125" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="D125" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
Tentando atualizar o orçamento
</commit_message>
<xml_diff>
--- a/3D/base_de_dados.xlsx
+++ b/3D/base_de_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PC- lixos\Downloads-24-11-2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1333BD21-C7BE-4974-9386-3C0D7AA2AB4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D643266F-BB0A-4029-915A-D692A600C454}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{F08DF800-D7FB-4182-BEE8-B029C50FA673}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="782" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="804" uniqueCount="326">
   <si>
     <t>CÓDIGO</t>
   </si>
@@ -985,6 +985,36 @@
   </si>
   <si>
     <t>CAIXA DE PASSAGEM PVC 4X2" - FORNECIMENTO E INSTALAÇÃO (COMPOSIÇÃO DE REFERÊNCIA: ORSE 777 - 06/2022)</t>
+  </si>
+  <si>
+    <t>Dispositivo de Proteção - Disjuntor bipolar termomagnético - 220 V/127 V - DIN - Curva C - 20 A - 5 kA</t>
+  </si>
+  <si>
+    <t>DISJUNTOR BIPOLAR TIPO DIN, CORRENTE NOMINAL DE 20A - FORNECIMENTO E INSTALAÇÃO. AF_07/2025</t>
+  </si>
+  <si>
+    <t>Dispositivo de Proteção - Disjuntor tripolar termomagnético - 220 V/127 V - DIN - Curva C - 100 A - 5 kA</t>
+  </si>
+  <si>
+    <t>Comp 128</t>
+  </si>
+  <si>
+    <t>DISJUNTOR TRIPOLAR TIPO DIN, CORRENTE NOMINAL DE 100A - FORNECIMENTO E INSTALAÇÃO. (COMPOSIÇÃO DE REFERÊNCIA: SINAPI 101895 - 04/2023)</t>
+  </si>
+  <si>
+    <t>Dispositivo de Proteção - Disjuntor tripolar termomagnético - 220 V/127 V - DIN - Curva C - 125 A - 40 kA</t>
+  </si>
+  <si>
+    <t>Comp 705</t>
+  </si>
+  <si>
+    <t>DISJUNTOR TRIPOLAR TIPO DIN, CORRENTE NOMINAL DE 125A - FORNECIMENTO E INSTALAÇÃO. AF_10/2020 (COMPOSIÇÃO REFERÊNCIA: SINAPI 93673)</t>
+  </si>
+  <si>
+    <t>Dispositivo de Comando - Relé fotoelétrico - fotocélula</t>
+  </si>
+  <si>
+    <t>RELÉ FOTOELÉTRICO PARA COMANDO DE ILUMINAÇÃO EXTERNA 1000 W - FORNECIMENTO E INSTALAÇÃO. AF_02/2025</t>
   </si>
 </sst>
 </file>
@@ -1371,7 +1401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A62C0A3C-3A73-4C24-9726-9CC231B21D7A}">
-  <dimension ref="A1:B141"/>
+  <dimension ref="A1:B145"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="96.77734375" style="3" bestFit="1" customWidth="1"/>
@@ -2162,7 +2192,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A99" s="3" t="s">
         <v>207</v>
       </c>
@@ -2322,7 +2352,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A119" s="3" t="s">
         <v>264</v>
       </c>
@@ -2503,6 +2533,38 @@
         <v>313</v>
       </c>
       <c r="B141" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A142" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="B142" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A143" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="B143" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A144" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="B144" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A145" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="B145" s="1" t="s">
         <v>7</v>
       </c>
     </row>
@@ -2513,7 +2575,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DACEE6F-7DD5-4F5D-8CC1-2F57EE446892}">
-  <dimension ref="A1:D141"/>
+  <dimension ref="A1:D145"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.109375" style="2" bestFit="1" customWidth="1"/>
@@ -4286,7 +4348,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A127" s="2" t="s">
         <v>279</v>
       </c>
@@ -4493,6 +4555,62 @@
         <v>315</v>
       </c>
       <c r="D141" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A142" s="2">
+        <v>93662</v>
+      </c>
+      <c r="B142" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C142" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="D142" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A143" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="B143" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C143" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="D143" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A144" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="B144" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C144" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="D144" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A145" s="2">
+        <v>101632</v>
+      </c>
+      <c r="B145" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C145" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="D145" s="2" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Tentando melhorar o orçamento
</commit_message>
<xml_diff>
--- a/3D/base_de_dados.xlsx
+++ b/3D/base_de_dados.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PC- lixos\Downloads-24-11-2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D643266F-BB0A-4029-915A-D692A600C454}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAE026E1-F517-4AF3-A79E-7EFEEA4A2202}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{F08DF800-D7FB-4182-BEE8-B029C50FA673}"/>
+    <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" xr2:uid="{F08DF800-D7FB-4182-BEE8-B029C50FA673}"/>
   </bookViews>
   <sheets>
     <sheet name="Associa" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="804" uniqueCount="326">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="836" uniqueCount="339">
   <si>
     <t>CÓDIGO</t>
   </si>
@@ -1015,6 +1015,45 @@
   </si>
   <si>
     <t>RELÉ FOTOELÉTRICO PARA COMANDO DE ILUMINAÇÃO EXTERNA 1000 W - FORNECIMENTO E INSTALAÇÃO. AF_02/2025</t>
+  </si>
+  <si>
+    <t>Dispositivo de Proteção - Disjuntor bipolar termomagnético - 220 V/127 V - DIN - Curva B - 20 A - 5 kA</t>
+  </si>
+  <si>
+    <t>Dispositivo de Proteção - Disjuntor bipolar termomagnético - 380 V/220 V - DIN - Curva C - 32 A - 25 kA</t>
+  </si>
+  <si>
+    <t>DISJUNTOR BIPOLAR TIPO DIN, CORRENTE NOMINAL DE 32A - FORNECIMENTO E INSTALAÇÃO. AF_07/2025</t>
+  </si>
+  <si>
+    <t>Lâmpadas Led - Luminária Pública - Lâmpada 120W</t>
+  </si>
+  <si>
+    <t>LUMINÁRIA DE LED PARA ILUMINAÇÃO PÚBLICA, DE 98 W ATÉ 137 W - FORNECIMENTO E INSTALAÇÃO. AF_02/2025_PS</t>
+  </si>
+  <si>
+    <t>Poste - Cônico em Aço Galvanizado - 7 metros</t>
+  </si>
+  <si>
+    <t>POSTE DE AÇO CÔNICO CONTÍNUO RETO, ENGASTAMENTO SIMPLES COM 1 M DE SOLO, H=7M - FORNECIMENTO E INSTALAÇÃO. AF_04/2025</t>
+  </si>
+  <si>
+    <t>Comp 1991</t>
+  </si>
+  <si>
+    <t>POSTE DE AÇO CONICO CONTÍNUO CURVO DUPLO, FLANGEADO, H=7M, INCLUSIVE LUMINÁRIAS, SEM LÂMPADAS - FORNECIMENTO E INSTALACAO. AF_11/2019  (COMPOSIÇÃO REFERÊNCIA: SINAPI 100621 08/2025)</t>
+  </si>
+  <si>
+    <t>Poste - Cônico duplo em Aço Galvanizado - 7 metros</t>
+  </si>
+  <si>
+    <t>Comp 1609</t>
+  </si>
+  <si>
+    <t>QUADRO DE DISTRIBUIÇÃO DE ENERGIA EM CHAPA DE AÇO GALVANIZADO, DE SOBREPOR, SEM BARRAMENTO, PARA 16 DISJUNTORES DIN - FORNECIMENTO E INSTALAÇÃO. AF_10/2020  (COMPOSIÇÃO REFERÊNCIA: SINAPI 101883)</t>
+  </si>
+  <si>
+    <t>Quadro distrib. chapa pintada - sobrepor - Sem barr., - DIN - Cap. 16 disj. unip.</t>
   </si>
 </sst>
 </file>
@@ -1401,7 +1440,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A62C0A3C-3A73-4C24-9726-9CC231B21D7A}">
-  <dimension ref="A1:B145"/>
+  <dimension ref="A1:B151"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="96.77734375" style="3" bestFit="1" customWidth="1"/>
@@ -2568,6 +2607,54 @@
         <v>7</v>
       </c>
     </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A146" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="B146" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A147" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="B147" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A148" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="B148" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A149" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="B149" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A150" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="B150" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A151" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="B151" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
@@ -2575,7 +2662,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DACEE6F-7DD5-4F5D-8CC1-2F57EE446892}">
-  <dimension ref="A1:D145"/>
+  <dimension ref="A1:D151"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.109375" style="2" bestFit="1" customWidth="1"/>
@@ -4614,6 +4701,90 @@
         <v>7</v>
       </c>
     </row>
+    <row r="146" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A146" s="2">
+        <v>93662</v>
+      </c>
+      <c r="B146" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C146" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="D146" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A147" s="2">
+        <v>93664</v>
+      </c>
+      <c r="B147" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C147" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="D147" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A148" s="2">
+        <v>101657</v>
+      </c>
+      <c r="B148" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C148" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="D148" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A149" s="2">
+        <v>105953</v>
+      </c>
+      <c r="B149" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C149" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="D149" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A150" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="B150" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C150" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="D150" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A151" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="B151" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C151" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="D151" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
Tentando melhorar as propriedades IFC
</commit_message>
<xml_diff>
--- a/3D/base_de_dados.xlsx
+++ b/3D/base_de_dados.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PC- lixos\Downloads-24-11-2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51A0EB51-E156-4EA6-841B-51E4EBFB668B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A72DE3D-770C-4F20-8AF8-752F13A4C6EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{F08DF800-D7FB-4182-BEE8-B029C50FA673}"/>
+    <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{F08DF800-D7FB-4182-BEE8-B029C50FA673}"/>
   </bookViews>
   <sheets>
     <sheet name="Associa" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="970" uniqueCount="392">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="986" uniqueCount="399">
   <si>
     <t>CÓDIGO</t>
   </si>
@@ -1213,6 +1213,27 @@
   </si>
   <si>
     <t>TE HORIZONTAL PARA ELETROCALHA 100X100MM (COMPOSIÇÃO DE REFERÊNCIA: SINAPI 97315 - 02/2023)</t>
+  </si>
+  <si>
+    <t>Acessórios p/ eletrodutos - Condulete alum. encaixe tipo LL - 1" sem tampa</t>
+  </si>
+  <si>
+    <t>Comp 1632</t>
+  </si>
+  <si>
+    <t>Acessórios p/ eletrodutos - Condulete alum. encaixe tipo LR - 1" sem tampa</t>
+  </si>
+  <si>
+    <t>Acessórios p/ eletrodutos - Condulete alum. encaixe tipo T - 1" sem tampa</t>
+  </si>
+  <si>
+    <t>CONDULETE DE ALUMÍNIO, TIPO LL, PARA ELETRODUTO DE AÇO GALVANIZADO DN 25 MM (1"), APARENTE - FORNECIMENTO E INSTALAÇÃO. AF_10/2022 (COMPOSIÇÃO REFERÊNCIA: SINAPI 95788 - 08/2025)</t>
+  </si>
+  <si>
+    <t>CONDULETE DE ALUMÍNIO, TIPO LR, PARA ELETRODUTO DE AÇO GALVANIZADO DN 25 MM (1"), APARENTE - FORNECIMENTO E INSTALAÇÃO. AF_01/2026</t>
+  </si>
+  <si>
+    <t>CONDULETE DE ALUMÍNIO, TIPO T, PARA ELETRODUTO DE AÇO GALVANIZADO DN 25 MM (1"), APARENTE - FORNECIMENTO E INSTALAÇÃO. AF_01/2026</t>
   </si>
 </sst>
 </file>
@@ -1599,7 +1620,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A62C0A3C-3A73-4C24-9726-9CC231B21D7A}">
-  <dimension ref="A1:B176"/>
+  <dimension ref="A1:B179"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="96.77734375" style="3" bestFit="1" customWidth="1"/>
@@ -3014,6 +3035,30 @@
         <v>7</v>
       </c>
     </row>
+    <row r="177" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A177" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="B177" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A178" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="B178" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A179" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="B179" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
@@ -3021,7 +3066,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DACEE6F-7DD5-4F5D-8CC1-2F57EE446892}">
-  <dimension ref="A1:D176"/>
+  <dimension ref="A1:D179"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.109375" style="2" bestFit="1" customWidth="1"/>
@@ -5494,6 +5539,48 @@
         <v>7</v>
       </c>
     </row>
+    <row r="177" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A177" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="B177" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C177" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="D177" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="178" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A178" s="2">
+        <v>95789</v>
+      </c>
+      <c r="B178" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C178" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="D178" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="179" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A179" s="2">
+        <v>95796</v>
+      </c>
+      <c r="B179" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C179" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="D179" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
Atualizando base de dados
</commit_message>
<xml_diff>
--- a/3D/base_de_dados.xlsx
+++ b/3D/base_de_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PC- lixos\Downloads-24-11-2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ABE975F-7A25-4B80-9324-0D0A52B2D592}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6722D4D5-EE99-4347-A0EF-1511838306DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{F08DF800-D7FB-4182-BEE8-B029C50FA673}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1247" uniqueCount="514">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1430" uniqueCount="563">
   <si>
     <t>CÓDIGO</t>
   </si>
@@ -1582,6 +1582,153 @@
   </si>
   <si>
     <t>CONECTOR SPLIT-BOLT, PARA SPDA, PARA CABOS DE 16 A 70 MM2 - FORNECIMENTO E INSTALAÇÃO. AF_08/2023 (COMPOSIÇÃO REFERÊNCIA: SINAPI 96982 01/2026)</t>
+  </si>
+  <si>
+    <t>.S.O.S CAIXA DE PASSAGEM - EMBUTIR NO PISO - Alvenaria - 30x30x30 cm</t>
+  </si>
+  <si>
+    <t>CAIXA ENTERRADA ELÉTRICA RETANGULAR, EM ALVENARIA COM TIJOLOS CERÂMICOS MACIÇOS, FUNDO COM BRITA, DIMENSÕES INTERNAS: 0,4X0,4X0,4 M. AF_12/2020</t>
+  </si>
+  <si>
+    <t>.S.O.S CAIXA DE PASSAGEM - EMBUTIR NO PISO - Alvenaria - 40x40x40 cm</t>
+  </si>
+  <si>
+    <t>.S.O.S CFTV e Segurança - NVR-PoE - 16 câmeras</t>
+  </si>
+  <si>
+    <t>Comp 652</t>
+  </si>
+  <si>
+    <t>NVR INTELBRAS 16 CANAIS FULL HD 1080P 2MP (COMPOSIÇÃO DE REFERÊNCIA: 068414 SBC 07/2024)</t>
+  </si>
+  <si>
+    <t>.S.O.S EQUIPAMENTOS DE TELECOMUNICAÇÕES - CABEAMENTO WIFI - Repetidor</t>
+  </si>
+  <si>
+    <t>Acessórios Cabeamento - Metálico - Bloco conexão - 110 IDC - 100 pares</t>
+  </si>
+  <si>
+    <t>Comp 532</t>
+  </si>
+  <si>
+    <t>BLOCO CONEXÃO - 110 IDC - 100 PARES (COMPOSIÇÃO DE REFERÊNCIA: SBC 059427 - 05/2023)</t>
+  </si>
+  <si>
+    <t>Acessórios Cabeamento - Metálico - Conector - RJ45 - Blindado</t>
+  </si>
+  <si>
+    <t>Acessórios Cabeamento - Metálico - Plugue - RJ45 - CM8v</t>
+  </si>
+  <si>
+    <t>Acessórios Cabeamento - Metálico - Switch - 10/100 - BaseTX - 24 portas</t>
+  </si>
+  <si>
+    <t>Comp 1612</t>
+  </si>
+  <si>
+    <t>SWITCH 24 - PORTAS (COMPOSIÇÃO DE REFERÊNCIA: SBC 059085 - 06/2022)</t>
+  </si>
+  <si>
+    <t>Acessórios Cabeamento - Rack - Bandeja de ventilação 1U - Kit 2 ventiladores - 400W</t>
+  </si>
+  <si>
+    <t>Comp 906</t>
+  </si>
+  <si>
+    <t>BANDEJA DE VENTILAÇÃO 1U COM 4 VENTILADORES - 400W. (REFERÊNCIA: SETOP ED-48376 10/2024)</t>
+  </si>
+  <si>
+    <t>Cabo Unipolar - cobre - Isol.PVC - 450/750V - ref. Pirastic Ecoplus BWF Flexível - 1.5 mm² - Amarelo</t>
+  </si>
+  <si>
+    <t>Cabo Unipolar - cobre - Isol.PVC - 450/750V - ref. Pirastic Ecoplus BWF Flexível - 1.5 mm² - Azul claro</t>
+  </si>
+  <si>
+    <t>Cabo Unipolar - cobre - Isol.PVC - 450/750V - ref. Pirastic Ecoplus BWF Flexível - 1.5 mm² - Preto</t>
+  </si>
+  <si>
+    <t>Cabo Unipolar - cobre - Isol.PVC - 450/750V - ref. Pirastic Ecoplus BWF Flexível - 1.5 mm² - Verde-amarelo</t>
+  </si>
+  <si>
+    <t>Cabo Unipolar - cobre - Isol.PVC - 450/750V - ref. Pirastic Ecoplus BWF Flexível - 1.5 mm² - Vermelho</t>
+  </si>
+  <si>
+    <t>CABO DE COBRE FLEXÍVEL ISOLADO, 1,5 MM², ANTI-CHAMA 450/750 V, PARA CIRCUITOS TERMINAIS - FORNECIMENTO E INSTALAÇÃO. AF_03/2023</t>
+  </si>
+  <si>
+    <t>Cabo Unipolar - cobre - Isol.PVC - 450/750V - ref. Pirastic Ecoplus BWF Flexível - 2.5 mm² - Amarelo</t>
+  </si>
+  <si>
+    <t>Cabo Unipolar - cobre - Isol.PVC - 450/750V - ref. Pirastic Ecoplus BWF Flexível - 2.5 mm² - Azul claro</t>
+  </si>
+  <si>
+    <t>Cabo Unipolar - cobre - Isol.PVC - 450/750V - ref. Pirastic Ecoplus BWF Flexível - 2.5 mm² - Branco</t>
+  </si>
+  <si>
+    <t>Cabo Unipolar - cobre - Isol.PVC - 450/750V - ref. Pirastic Ecoplus BWF Flexível - 2.5 mm² - Preto</t>
+  </si>
+  <si>
+    <t>Cabo Unipolar - cobre - Isol.PVC - 450/750V - ref. Pirastic Ecoplus BWF Flexível - 2.5 mm² - Verde-amarelo</t>
+  </si>
+  <si>
+    <t>Cabo Unipolar - cobre - Isol.PVC - 450/750V - ref. Pirastic Ecoplus BWF Flexível - 2.5 mm² - Vermelho</t>
+  </si>
+  <si>
+    <t>CABO DE COBRE FLEXÍVEL ISOLADO, 2,5 MM², ANTI-CHAMA 450/750 V, PARA CIRCUITOS TERMINAIS - FORNECIMENTO E INSTALAÇÃO. AF_03/2023</t>
+  </si>
+  <si>
+    <t>Cabo Unipolar - cobre - Isol.PVC - 450/750V - ref. Pirastic Ecoplus BWF Flexível - 4 mm² - Azul claro</t>
+  </si>
+  <si>
+    <t>Cabo Unipolar - cobre - Isol.PVC - 450/750V - ref. Pirastic Ecoplus BWF Flexível - 4 mm² - Preto</t>
+  </si>
+  <si>
+    <t>Cabo Unipolar - cobre - Isol.PVC - 450/750V - ref. Pirastic Ecoplus BWF Flexível - 4 mm² - Verde-amarelo</t>
+  </si>
+  <si>
+    <t>Cabo Unipolar - cobre - Isol.PVC - 450/750V - ref. Pirastic Ecoplus BWF Flexível - 4 mm² - Vermelho</t>
+  </si>
+  <si>
+    <t>CABO DE COBRE FLEXÍVEL ISOLADO, 4 MM², ANTI-CHAMA 450/750 V, PARA CIRCUITOS TERMINAIS - FORNECIMENTO E INSTALAÇÃO. AF_03/2023</t>
+  </si>
+  <si>
+    <t>Cabo Unipolar - cobre - Isol.PVC - 450/750V - ref. Pirastic Ecoplus BWF Flexível - 16 mm² - Branco</t>
+  </si>
+  <si>
+    <t>Cabo Unipolar - cobre - Isol.PVC - 450/750V - ref. Pirastic Ecoplus BWF Flexível - 16 mm² - Preto</t>
+  </si>
+  <si>
+    <t>Cabo Unipolar - cobre - Isol.PVC - 450/750V - ref. Pirastic Ecoplus BWF Flexível - 16 mm² - Verde-amarelo</t>
+  </si>
+  <si>
+    <t>Cabo Unipolar - cobre - Isol.PVC - 450/750V - ref. Pirastic Ecoplus BWF Flexível - 16 mm² - Vermelho</t>
+  </si>
+  <si>
+    <t>CABO DE COBRE FLEXÍVEL ISOLADO, 16 MM², ANTI-CHAMA 450/750 V, PARA CIRCUITOS TERMINAIS - FORNECIMENTO E INSTALAÇÃO. AF_03/2023</t>
+  </si>
+  <si>
+    <t>Cabo - Plugue - Plugue fêmea</t>
+  </si>
+  <si>
+    <t>Cabeamento estruturado - metálico - UTP-5e - 24AWG - 4</t>
+  </si>
+  <si>
+    <t>CABO ELETRÔNICO CATEGORIA 5E, INSTALADO EM EDIFICAÇÃO INSTITUCIONAL - FORNECIMENTO E INSTALAÇÃO. AF_08/2025</t>
+  </si>
+  <si>
+    <t>Cabo Unipolar - cobre - Isol. XLPE - 0,6/1kV - ref. Prysmian Voltalene Ecolene - 16 mm² - Verde-amarelo</t>
+  </si>
+  <si>
+    <t>Cabo Unipolar - cobre - Isol. XLPE - 0,6/1kV - ref. Prysmian Voltalene Ecolene - 25 mm² - Azul claro</t>
+  </si>
+  <si>
+    <t>Cabo Unipolar - cobre - Isol. XLPE - 0,6/1kV - ref. Prysmian Voltalene Ecolene - 25 mm² - Branco</t>
+  </si>
+  <si>
+    <t>Cabo Unipolar - cobre - Isol. XLPE - 0,6/1kV - ref. Prysmian Voltalene Ecolene - 25 mm² - Preto</t>
+  </si>
+  <si>
+    <t>Cabo Unipolar - cobre - Isol. XLPE - 0,6/1kV - ref. Prysmian Voltalene Ecolene - 25 mm² - Vermelho</t>
   </si>
 </sst>
 </file>
@@ -1968,7 +2115,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A62C0A3C-3A73-4C24-9726-9CC231B21D7A}">
-  <dimension ref="A1:B226"/>
+  <dimension ref="A1:B261"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="96.77734375" style="3" bestFit="1" customWidth="1"/>
@@ -3783,6 +3930,286 @@
         <v>7</v>
       </c>
     </row>
+    <row r="227" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A227" s="3" t="s">
+        <v>514</v>
+      </c>
+      <c r="B227" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A228" s="3" t="s">
+        <v>516</v>
+      </c>
+      <c r="B228" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="229" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A229" s="3" t="s">
+        <v>517</v>
+      </c>
+      <c r="B229" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="230" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A230" s="3" t="s">
+        <v>520</v>
+      </c>
+      <c r="B230" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A231" s="3" t="s">
+        <v>521</v>
+      </c>
+      <c r="B231" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="232" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A232" s="3" t="s">
+        <v>524</v>
+      </c>
+      <c r="B232" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="233" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A233" s="3" t="s">
+        <v>525</v>
+      </c>
+      <c r="B233" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="234" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A234" s="3" t="s">
+        <v>526</v>
+      </c>
+      <c r="B234" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="235" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A235" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="B235" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="236" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A236" s="3" t="s">
+        <v>532</v>
+      </c>
+      <c r="B236" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="237" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A237" s="3" t="s">
+        <v>533</v>
+      </c>
+      <c r="B237" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="238" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A238" s="3" t="s">
+        <v>534</v>
+      </c>
+      <c r="B238" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="239" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A239" s="3" t="s">
+        <v>535</v>
+      </c>
+      <c r="B239" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="240" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A240" s="3" t="s">
+        <v>536</v>
+      </c>
+      <c r="B240" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="241" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A241" s="3" t="s">
+        <v>538</v>
+      </c>
+      <c r="B241" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="242" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A242" s="3" t="s">
+        <v>539</v>
+      </c>
+      <c r="B242" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="243" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A243" s="3" t="s">
+        <v>540</v>
+      </c>
+      <c r="B243" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="244" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A244" s="3" t="s">
+        <v>541</v>
+      </c>
+      <c r="B244" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="245" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A245" s="3" t="s">
+        <v>542</v>
+      </c>
+      <c r="B245" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="246" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A246" s="3" t="s">
+        <v>543</v>
+      </c>
+      <c r="B246" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="247" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A247" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="B247" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="248" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A248" s="3" t="s">
+        <v>546</v>
+      </c>
+      <c r="B248" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="249" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A249" s="3" t="s">
+        <v>547</v>
+      </c>
+      <c r="B249" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="250" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A250" s="3" t="s">
+        <v>548</v>
+      </c>
+      <c r="B250" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="251" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A251" s="3" t="s">
+        <v>550</v>
+      </c>
+      <c r="B251" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="252" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A252" s="3" t="s">
+        <v>551</v>
+      </c>
+      <c r="B252" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="253" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A253" s="3" t="s">
+        <v>552</v>
+      </c>
+      <c r="B253" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="254" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A254" s="3" t="s">
+        <v>553</v>
+      </c>
+      <c r="B254" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="255" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A255" s="3" t="s">
+        <v>555</v>
+      </c>
+      <c r="B255" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="256" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A256" s="3" t="s">
+        <v>556</v>
+      </c>
+      <c r="B256" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="257" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A257" s="3" t="s">
+        <v>558</v>
+      </c>
+      <c r="B257" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="258" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A258" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="B258" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="259" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A259" s="3" t="s">
+        <v>560</v>
+      </c>
+      <c r="B259" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="260" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A260" s="3" t="s">
+        <v>561</v>
+      </c>
+      <c r="B260" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="261" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A261" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="B261" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
@@ -3790,7 +4217,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DACEE6F-7DD5-4F5D-8CC1-2F57EE446892}">
-  <dimension ref="A1:D226"/>
+  <dimension ref="A1:D261"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.109375" style="2" bestFit="1" customWidth="1"/>
@@ -6963,6 +7390,496 @@
         <v>7</v>
       </c>
     </row>
+    <row r="227" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A227" s="2">
+        <v>97886</v>
+      </c>
+      <c r="B227" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C227" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="D227" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="228" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A228" s="2">
+        <v>97887</v>
+      </c>
+      <c r="B228" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C228" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="D228" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="229" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A229" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="B229" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C229" s="3" t="s">
+        <v>519</v>
+      </c>
+      <c r="D229" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="230" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A230" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="B230" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C230" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="D230" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="231" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A231" s="2" t="s">
+        <v>522</v>
+      </c>
+      <c r="B231" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C231" s="3" t="s">
+        <v>523</v>
+      </c>
+      <c r="D231" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="232" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A232" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="B232" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C232" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="D232" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="233" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A233" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B233" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C233" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="D233" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="234" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A234" s="2" t="s">
+        <v>527</v>
+      </c>
+      <c r="B234" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C234" s="3" t="s">
+        <v>528</v>
+      </c>
+      <c r="D234" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="235" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A235" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="B235" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C235" s="3" t="s">
+        <v>531</v>
+      </c>
+      <c r="D235" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="236" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A236" s="2">
+        <v>91924</v>
+      </c>
+      <c r="B236" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C236" s="3" t="s">
+        <v>537</v>
+      </c>
+      <c r="D236" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="237" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A237" s="2">
+        <v>91924</v>
+      </c>
+      <c r="B237" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C237" s="3" t="s">
+        <v>537</v>
+      </c>
+      <c r="D237" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="238" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A238" s="2">
+        <v>91924</v>
+      </c>
+      <c r="B238" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C238" s="3" t="s">
+        <v>537</v>
+      </c>
+      <c r="D238" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="239" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A239" s="2">
+        <v>91924</v>
+      </c>
+      <c r="B239" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C239" s="3" t="s">
+        <v>537</v>
+      </c>
+      <c r="D239" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="240" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A240" s="2">
+        <v>91924</v>
+      </c>
+      <c r="B240" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C240" s="3" t="s">
+        <v>537</v>
+      </c>
+      <c r="D240" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="241" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A241" s="2">
+        <v>91926</v>
+      </c>
+      <c r="B241" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C241" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="D241" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="242" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A242" s="2">
+        <v>91926</v>
+      </c>
+      <c r="B242" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C242" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="D242" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="243" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A243" s="2">
+        <v>91926</v>
+      </c>
+      <c r="B243" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C243" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="D243" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="244" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A244" s="2">
+        <v>91926</v>
+      </c>
+      <c r="B244" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C244" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="D244" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="245" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A245" s="2">
+        <v>91926</v>
+      </c>
+      <c r="B245" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C245" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="D245" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="246" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A246" s="2">
+        <v>91926</v>
+      </c>
+      <c r="B246" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C246" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="D246" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="247" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A247" s="2">
+        <v>91928</v>
+      </c>
+      <c r="B247" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C247" s="3" t="s">
+        <v>549</v>
+      </c>
+      <c r="D247" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="248" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A248" s="2">
+        <v>91928</v>
+      </c>
+      <c r="B248" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C248" s="3" t="s">
+        <v>549</v>
+      </c>
+      <c r="D248" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="249" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A249" s="2">
+        <v>91928</v>
+      </c>
+      <c r="B249" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C249" s="3" t="s">
+        <v>549</v>
+      </c>
+      <c r="D249" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="250" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A250" s="2">
+        <v>91928</v>
+      </c>
+      <c r="B250" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C250" s="3" t="s">
+        <v>549</v>
+      </c>
+      <c r="D250" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="251" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A251" s="2">
+        <v>91934</v>
+      </c>
+      <c r="B251" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C251" s="3" t="s">
+        <v>554</v>
+      </c>
+      <c r="D251" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="252" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A252" s="2">
+        <v>91934</v>
+      </c>
+      <c r="B252" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C252" s="3" t="s">
+        <v>554</v>
+      </c>
+      <c r="D252" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="253" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A253" s="2">
+        <v>91934</v>
+      </c>
+      <c r="B253" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C253" s="3" t="s">
+        <v>554</v>
+      </c>
+      <c r="D253" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="254" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A254" s="2">
+        <v>91934</v>
+      </c>
+      <c r="B254" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C254" s="3" t="s">
+        <v>554</v>
+      </c>
+      <c r="D254" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="255" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A255" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B255" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C255" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D255" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="256" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A256" s="2">
+        <v>98295</v>
+      </c>
+      <c r="B256" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C256" s="3" t="s">
+        <v>557</v>
+      </c>
+      <c r="D256" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="257" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A257" s="2">
+        <v>91935</v>
+      </c>
+      <c r="B257" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C257" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D257" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="258" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A258" s="2">
+        <v>92984</v>
+      </c>
+      <c r="B258" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C258" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D258" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="259" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A259" s="2">
+        <v>92984</v>
+      </c>
+      <c r="B259" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C259" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D259" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="260" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A260" s="2">
+        <v>92984</v>
+      </c>
+      <c r="B260" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C260" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D260" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="261" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A261" s="2">
+        <v>92984</v>
+      </c>
+      <c r="B261" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C261" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D261" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D226" xr:uid="{8DACEE6F-7DD5-4F5D-8CC1-2F57EE446892}"/>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>